<commit_message>
Update asset report to use correct preload value setting
Corrected the "Preload" setting key to "FlowPreloadCharge" in the ewater API routes and updated the asset report title.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: aa2546f1-ca0a-4a81-a77c-96757e0feb86
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b1ff869f-74ed-4a0b-af06-a3d77aba0810
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/45976032-64bc-43ca-901d-c81de5c4ad70/aa2546f1-ca0a-4a81-a77c-96757e0feb86/H1OQ6h1
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/Ol_Moran_Asset_Report.xlsx
+++ b/exports/Ol_Moran_Asset_Report.xlsx
@@ -527,7 +527,9 @@
       <c r="F2" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="G2" s="3" t="n"/>
+      <c r="G2" s="3" t="n">
+        <v>365</v>
+      </c>
       <c r="H2" s="3" t="n">
         <v>22.05</v>
       </c>
@@ -557,7 +559,9 @@
       <c r="F3" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="G3" s="3" t="n"/>
+      <c r="G3" s="3" t="n">
+        <v>365</v>
+      </c>
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n">
@@ -579,21 +583,21 @@
         <v>2105</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>52.45</v>
+        <v>52.31</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>29.68</v>
+        <v>29.75</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="n">
-        <v>28.95</v>
+        <v>28.85</v>
       </c>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +623,9 @@
       <c r="F5" s="3" t="n">
         <v>382</v>
       </c>
-      <c r="G5" s="3" t="n"/>
+      <c r="G5" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H5" s="3" t="n">
         <v>18.85</v>
       </c>
@@ -653,7 +659,9 @@
       <c r="F6" s="3" t="n">
         <v>375</v>
       </c>
-      <c r="G6" s="3" t="n"/>
+      <c r="G6" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H6" s="3" t="n">
         <v>17.6</v>
       </c>
@@ -687,7 +695,9 @@
       <c r="F7" s="3" t="n">
         <v>358</v>
       </c>
-      <c r="G7" s="3" t="n"/>
+      <c r="G7" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H7" s="3" t="n">
         <v>22.1</v>
       </c>
@@ -721,7 +731,9 @@
       <c r="F8" s="3" t="n">
         <v>373</v>
       </c>
-      <c r="G8" s="3" t="n"/>
+      <c r="G8" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H8" s="3" t="n">
         <v>16.55</v>
       </c>
@@ -755,7 +767,9 @@
       <c r="F9" s="3" t="n">
         <v>389</v>
       </c>
-      <c r="G9" s="3" t="n"/>
+      <c r="G9" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H9" s="3" t="n">
         <v>10.95</v>
       </c>
@@ -789,7 +803,9 @@
       <c r="F10" s="3" t="n">
         <v>369</v>
       </c>
-      <c r="G10" s="3" t="n"/>
+      <c r="G10" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H10" s="3" t="n">
         <v>22.4</v>
       </c>
@@ -823,7 +839,9 @@
       <c r="F11" s="3" t="n">
         <v>381</v>
       </c>
-      <c r="G11" s="3" t="n"/>
+      <c r="G11" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H11" s="3" t="n">
         <v>19.55</v>
       </c>
@@ -857,7 +875,9 @@
       <c r="F12" s="3" t="n">
         <v>428</v>
       </c>
-      <c r="G12" s="3" t="n"/>
+      <c r="G12" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n">
@@ -887,7 +907,9 @@
       <c r="F13" s="3" t="n">
         <v>354</v>
       </c>
-      <c r="G13" s="3" t="n"/>
+      <c r="G13" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H13" s="3" t="n">
         <v>19.55</v>
       </c>
@@ -921,7 +943,9 @@
       <c r="F14" s="3" t="n">
         <v>348</v>
       </c>
-      <c r="G14" s="3" t="n"/>
+      <c r="G14" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H14" s="3" t="n">
         <v>21.75</v>
       </c>
@@ -955,7 +979,9 @@
       <c r="F15" s="3" t="n">
         <v>375</v>
       </c>
-      <c r="G15" s="3" t="n"/>
+      <c r="G15" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H15" s="3" t="n">
         <v>22.4</v>
       </c>
@@ -989,7 +1015,9 @@
       <c r="F16" s="3" t="n">
         <v>369</v>
       </c>
-      <c r="G16" s="3" t="n"/>
+      <c r="G16" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H16" s="3" t="n">
         <v>20.4</v>
       </c>
@@ -1023,7 +1051,9 @@
       <c r="F17" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="G17" s="3" t="n"/>
+      <c r="G17" s="3" t="n">
+        <v>365</v>
+      </c>
       <c r="H17" s="3" t="n">
         <v>19.6</v>
       </c>
@@ -1057,7 +1087,9 @@
       <c r="F18" s="3" t="n">
         <v>392</v>
       </c>
-      <c r="G18" s="3" t="n"/>
+      <c r="G18" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H18" s="3" t="n">
         <v>28.8</v>
       </c>
@@ -1089,7 +1121,9 @@
       <c r="F19" s="3" t="n">
         <v>368</v>
       </c>
-      <c r="G19" s="3" t="n"/>
+      <c r="G19" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H19" s="3" t="n">
         <v>19.3</v>
       </c>
@@ -1123,7 +1157,9 @@
       <c r="F20" s="3" t="n">
         <v>385</v>
       </c>
-      <c r="G20" s="3" t="n"/>
+      <c r="G20" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H20" s="3" t="n">
         <v>18.45</v>
       </c>
@@ -1157,7 +1193,9 @@
       <c r="F21" s="3" t="n">
         <v>379</v>
       </c>
-      <c r="G21" s="3" t="n"/>
+      <c r="G21" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H21" s="3" t="n">
         <v>20.35</v>
       </c>
@@ -1191,7 +1229,9 @@
       <c r="F22" s="3" t="n">
         <v>362</v>
       </c>
-      <c r="G22" s="3" t="n"/>
+      <c r="G22" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H22" s="3" t="n">
         <v>18.25</v>
       </c>
@@ -1225,7 +1265,9 @@
       <c r="F23" s="3" t="n">
         <v>344</v>
       </c>
-      <c r="G23" s="3" t="n"/>
+      <c r="G23" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n">
@@ -1255,7 +1297,9 @@
       <c r="F24" s="3" t="n">
         <v>382</v>
       </c>
-      <c r="G24" s="3" t="n"/>
+      <c r="G24" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H24" s="3" t="n">
         <v>19</v>
       </c>
@@ -1289,7 +1333,9 @@
       <c r="F25" s="3" t="n">
         <v>390</v>
       </c>
-      <c r="G25" s="3" t="n"/>
+      <c r="G25" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H25" s="3" t="n">
         <v>17.85</v>
       </c>
@@ -1323,7 +1369,9 @@
       <c r="F26" s="3" t="n">
         <v>365</v>
       </c>
-      <c r="G26" s="3" t="n"/>
+      <c r="G26" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H26" s="3" t="n">
         <v>17.1</v>
       </c>
@@ -1357,7 +1405,9 @@
       <c r="F27" s="3" t="n">
         <v>381</v>
       </c>
-      <c r="G27" s="3" t="n"/>
+      <c r="G27" s="3" t="n">
+        <v>400</v>
+      </c>
       <c r="H27" s="3" t="n">
         <v>20.35</v>
       </c>

</xml_diff>